<commit_message>
Update BarrelIQ live data
</commit_message>
<xml_diff>
--- a/outputs/daily/hr_rankings_2026-10-01.xlsx
+++ b/outputs/daily/hr_rankings_2026-10-01.xlsx
@@ -760,7 +760,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -6686,7 +6686,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -6966,7 +6966,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -7526,7 +7526,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -8366,7 +8366,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -8926,7 +8926,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -9206,7 +9206,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -9486,7 +9486,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -9766,7 +9766,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -10046,7 +10046,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -10326,7 +10326,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">

</xml_diff>